<commit_message>
Rename tournament tabs and package TOAST only
</commit_message>
<xml_diff>
--- a/2026-FLL-Qualifier-Tournaments-with-divisions.xlsx
+++ b/2026-FLL-Qualifier-Tournaments-with-divisions.xlsx
@@ -14,8 +14,8 @@
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="9" r:id="rId1"/>
-    <sheet name="Tournaments" sheetId="7" r:id="rId2"/>
-    <sheet name="DivTournaments" sheetId="11" r:id="rId3"/>
+    <sheet name="Single Division" sheetId="7" r:id="rId2"/>
+    <sheet name="Two Divisions" sheetId="11" r:id="rId3"/>
     <sheet name="Assignments" sheetId="8" r:id="rId4"/>
     <sheet name="SeasonInfo" sheetId="12" r:id="rId5"/>
     <sheet name="AwardDef" sheetId="13" r:id="rId6"/>
@@ -4989,7 +4989,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Putting an award on this sheet does not automatically mean it will appear in any given tournament OJS. That is determined by how many of those awards are allocated for each tournament on the Tournaments worksheet and DivAwards worksheet. This worksheet only defines the award. If you list an award here that has 0 allocations at any and all tournaments, that award will not show up on any OJS. This is only a lookup table to get the definition for an award</a:t>
+            <a:t>Putting an award on this sheet does not automatically mean it will appear in any given tournament OJS. That is determined by how many of those awards are allocated for each tournament on the Single Division worksheet and Two Divisions worksheet. This worksheet only defines the award. If you list an award here that has 0 allocations at any and all tournaments, that award will not show up on any OJS. This is only a lookup table to get the definition for an award</a:t>
           </a:r>
           <a:endParaRPr lang="en-US">
             <a:effectLst/>
@@ -5001,7 +5001,7 @@
         <a:p>
           <a:r>
             <a:rPr lang="en-US" sz="1100"/>
-            <a:t>For ColumnName, enter in the column name as used on the Tournaments and DivAwards worksheets.</a:t>
+            <a:t>For ColumnName, enter in the column name as used on the Single Division and Two Divisions worksheets.</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" baseline="0"/>

</xml_diff>